<commit_message>
feat: clarify product and demonstrate Coze workflow
</commit_message>
<xml_diff>
--- a/collaboration/integration/final_outputs/ready_to_use/05_资源索引/统一交付资源索引.xlsx
+++ b/collaboration/integration/final_outputs/ready_to_use/05_资源索引/统一交付资源索引.xlsx
@@ -2251,7 +2251,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>DOCX_五套样例端到端验收_20260718_170906.json</t>
+          <t>DOCX_五套样例端到端验收_20260718_174546.json</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -2264,12 +2264,12 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>0dc9ca9f4a567d2c1571949c5bf960eef7a2e83471fda005ce8c0b8b85ce6bca</t>
+          <t>9c939f2628d581b5d43bfeb0ac5b5f2a21fc312b1a41cbf3fc1cd326bb385a6b</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX_五套样例端到端验收_20260718_170906.json</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX_五套样例端到端验收_20260718_174546.json</t>
         </is>
       </c>
     </row>
@@ -2281,7 +2281,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试1_20260718_170905.docx</t>
+          <t>DOCX样例_测试1_20260718_174545.docx</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -2299,7 +2299,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试1_20260718_170905.docx</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试1_20260718_174545.docx</t>
         </is>
       </c>
     </row>
@@ -2311,7 +2311,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试1_20260718_170905.回填报告.json</t>
+          <t>DOCX样例_测试1_20260718_174545.回填报告.json</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -2324,12 +2324,12 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>ddcc436c212c8aef27f903bc891306289e712420a73239b0b11eb85f962ab3e5</t>
+          <t>abb56588736a7865f407148229c1a795a931d12b9b565370c522d55ce884390e</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试1_20260718_170905.回填报告.json</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试1_20260718_174545.回填报告.json</t>
         </is>
       </c>
     </row>
@@ -2341,7 +2341,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试2_20260718_170905.docx</t>
+          <t>DOCX样例_测试2_20260718_174546.docx</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -2359,7 +2359,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试2_20260718_170905.docx</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试2_20260718_174546.docx</t>
         </is>
       </c>
     </row>
@@ -2371,7 +2371,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试2_20260718_170905.回填报告.json</t>
+          <t>DOCX样例_测试2_20260718_174546.回填报告.json</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -2384,12 +2384,12 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>29f00c718974b514f9def4378699225b170df0cef6366be3284c798fe1ca6038</t>
+          <t>a3654879e1083771794b3e2dbd42aae0ae0bfdc4ba4196326d6896fd60175d16</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试2_20260718_170905.回填报告.json</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试2_20260718_174546.回填报告.json</t>
         </is>
       </c>
     </row>
@@ -2401,7 +2401,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试3_20260718_170905.docx</t>
+          <t>DOCX样例_测试3_20260718_174546.docx</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试3_20260718_170905.docx</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试3_20260718_174546.docx</t>
         </is>
       </c>
     </row>
@@ -2431,7 +2431,7 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试3_20260718_170905.回填报告.json</t>
+          <t>DOCX样例_测试3_20260718_174546.回填报告.json</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -2444,12 +2444,12 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>37876550ed51d686dfb420f59f6681c3335a00ab194032cb7236cf408d67d4fc</t>
+          <t>b79f630ac8935763ad6eefd61942285510d4285455ecd5449fa0c8f9741e3f36</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试3_20260718_170905.回填报告.json</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试3_20260718_174546.回填报告.json</t>
         </is>
       </c>
     </row>
@@ -2461,7 +2461,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试4_20260718_170906.docx</t>
+          <t>DOCX样例_测试4_20260718_174546.docx</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -2479,7 +2479,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试4_20260718_170906.docx</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试4_20260718_174546.docx</t>
         </is>
       </c>
     </row>
@@ -2491,7 +2491,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试4_20260718_170906.回填报告.json</t>
+          <t>DOCX样例_测试4_20260718_174546.回填报告.json</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -2504,12 +2504,12 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>759d03ac5baa531ece1cca6587b934ba79298d152caaad41d7fd6a6a6c2577c5</t>
+          <t>e691a6b8b90dbf504e85c197619dfed89de4373ae6d0c125aa52c59a912b06f6</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试4_20260718_170906.回填报告.json</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试4_20260718_174546.回填报告.json</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试5_20260718_170906.docx</t>
+          <t>DOCX样例_测试5_20260718_174546.docx</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -2539,7 +2539,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试5_20260718_170906.docx</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试5_20260718_174546.docx</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试5_20260718_170906.回填报告.json</t>
+          <t>DOCX样例_测试5_20260718_174546.回填报告.json</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -2564,12 +2564,12 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>7958f9a5b778a3a5c1122f0f6433e75c297f192eeae38c63df639fe5246ea117</t>
+          <t>45d4c85d93087b4a9592b57f666f56a84146d08732089e6716f0a41dba7c657d</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试5_20260718_170906.回填报告.json</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试5_20260718_174546.回填报告.json</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_170906.txt</t>
+          <t>translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_174546.txt</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -2839,7 +2839,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>04_音视频翻译/本机重新生成产出/translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_170906.txt</t>
+          <t>04_音视频翻译/本机重新生成产出/translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_174546.txt</t>
         </is>
       </c>
     </row>
@@ -2851,7 +2851,7 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_170906.wav</t>
+          <t>translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_174546.wav</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -2869,7 +2869,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>04_音视频翻译/本机重新生成产出/translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_170906.wav</t>
+          <t>04_音视频翻译/本机重新生成产出/translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_174546.wav</t>
         </is>
       </c>
     </row>
@@ -2881,7 +2881,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_170906.二维码.png</t>
+          <t>translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_174546.二维码.png</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -2890,16 +2890,16 @@
         </is>
       </c>
       <c r="D82" s="2" t="n">
-        <v>2516</v>
+        <v>2500</v>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>8bdb5a2169b274e7f06058f3bf9ce8a726d2effb29c8580637ef186e5f5d2378</t>
+          <t>c8b13de714f8fda66f78ad2d103cf3fdaa771b4a3d1a1475e7d934f78de98d92</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>04_音视频翻译/本机重新生成产出/translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_170906.二维码.png</t>
+          <t>04_音视频翻译/本机重新生成产出/translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_174546.二维码.png</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: rebrand as Yishu and refine desktop experience
</commit_message>
<xml_diff>
--- a/collaboration/integration/final_outputs/ready_to_use/05_资源索引/统一交付资源索引.xlsx
+++ b/collaboration/integration/final_outputs/ready_to_use/05_资源索引/统一交付资源索引.xlsx
@@ -2251,7 +2251,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>DOCX_五套样例端到端验收_20260718_174546.json</t>
+          <t>DOCX_五套样例端到端验收_20260718_194336.json</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -2264,12 +2264,12 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>9c939f2628d581b5d43bfeb0ac5b5f2a21fc312b1a41cbf3fc1cd326bb385a6b</t>
+          <t>e3b1cd17bec39223987162d78b17f4a2aeb7a3c0e32ab66bcd1ccb01daefdafd</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX_五套样例端到端验收_20260718_174546.json</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX_五套样例端到端验收_20260718_194336.json</t>
         </is>
       </c>
     </row>
@@ -2281,7 +2281,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试1_20260718_174545.docx</t>
+          <t>DOCX样例_测试1_20260718_194336.docx</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -2299,7 +2299,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试1_20260718_174545.docx</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试1_20260718_194336.docx</t>
         </is>
       </c>
     </row>
@@ -2311,7 +2311,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试1_20260718_174545.回填报告.json</t>
+          <t>DOCX样例_测试1_20260718_194336.回填报告.json</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -2324,12 +2324,12 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>abb56588736a7865f407148229c1a795a931d12b9b565370c522d55ce884390e</t>
+          <t>62e78b877bf03de379bc58eb32c33515ff80a420e2019f3c56f0a8221a827096</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试1_20260718_174545.回填报告.json</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试1_20260718_194336.回填报告.json</t>
         </is>
       </c>
     </row>
@@ -2341,7 +2341,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试2_20260718_174546.docx</t>
+          <t>DOCX样例_测试2_20260718_194336.docx</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -2359,7 +2359,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试2_20260718_174546.docx</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试2_20260718_194336.docx</t>
         </is>
       </c>
     </row>
@@ -2371,7 +2371,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试2_20260718_174546.回填报告.json</t>
+          <t>DOCX样例_测试2_20260718_194336.回填报告.json</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -2384,12 +2384,12 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>a3654879e1083771794b3e2dbd42aae0ae0bfdc4ba4196326d6896fd60175d16</t>
+          <t>46ee547d2836fb99d84258402e50bdda4ae58cfe4e1c9ee5ca13c2e36d7ea076</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试2_20260718_174546.回填报告.json</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试2_20260718_194336.回填报告.json</t>
         </is>
       </c>
     </row>
@@ -2401,7 +2401,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试3_20260718_174546.docx</t>
+          <t>DOCX样例_测试3_20260718_194336.docx</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试3_20260718_174546.docx</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试3_20260718_194336.docx</t>
         </is>
       </c>
     </row>
@@ -2431,7 +2431,7 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试3_20260718_174546.回填报告.json</t>
+          <t>DOCX样例_测试3_20260718_194336.回填报告.json</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -2444,12 +2444,12 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>b79f630ac8935763ad6eefd61942285510d4285455ecd5449fa0c8f9741e3f36</t>
+          <t>b94b1d90644287c1a88c33a5c58797f3fb6fcab57c5e84eb7f7d39185400cd4f</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试3_20260718_174546.回填报告.json</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试3_20260718_194336.回填报告.json</t>
         </is>
       </c>
     </row>
@@ -2461,7 +2461,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试4_20260718_174546.docx</t>
+          <t>DOCX样例_测试4_20260718_194336.docx</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -2479,7 +2479,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试4_20260718_174546.docx</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试4_20260718_194336.docx</t>
         </is>
       </c>
     </row>
@@ -2491,7 +2491,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试4_20260718_174546.回填报告.json</t>
+          <t>DOCX样例_测试4_20260718_194336.回填报告.json</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -2504,12 +2504,12 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>e691a6b8b90dbf504e85c197619dfed89de4373ae6d0c125aa52c59a912b06f6</t>
+          <t>76c97f70d0c3966a075e55cad784c198559f254d3dd78db40328ea8de054baaf</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试4_20260718_174546.回填报告.json</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试4_20260718_194336.回填报告.json</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试5_20260718_174546.docx</t>
+          <t>DOCX样例_测试5_20260718_194336.docx</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -2539,7 +2539,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试5_20260718_174546.docx</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试5_20260718_194336.docx</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试5_20260718_174546.回填报告.json</t>
+          <t>DOCX样例_测试5_20260718_194336.回填报告.json</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -2564,12 +2564,12 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>45d4c85d93087b4a9592b57f666f56a84146d08732089e6716f0a41dba7c657d</t>
+          <t>6d599971c03ef0c796f8e91dd3d11f928045711a8b5dcc7423f4d869c4ac2197</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试5_20260718_174546.回填报告.json</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试5_20260718_194336.回填报告.json</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_174546.txt</t>
+          <t>translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_194336.txt</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -2839,7 +2839,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>04_音视频翻译/本机重新生成产出/translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_174546.txt</t>
+          <t>04_音视频翻译/本机重新生成产出/translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_194336.txt</t>
         </is>
       </c>
     </row>
@@ -2851,7 +2851,7 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_174546.wav</t>
+          <t>translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_194336.wav</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -2869,7 +2869,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>04_音视频翻译/本机重新生成产出/translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_174546.wav</t>
+          <t>04_音视频翻译/本机重新生成产出/translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_194336.wav</t>
         </is>
       </c>
     </row>
@@ -2881,7 +2881,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_174546.二维码.png</t>
+          <t>translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_194336.二维码.png</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -2890,16 +2890,16 @@
         </is>
       </c>
       <c r="D82" s="2" t="n">
-        <v>2500</v>
+        <v>2523</v>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>c8b13de714f8fda66f78ad2d103cf3fdaa771b4a3d1a1475e7d934f78de98d92</t>
+          <t>b367e1b6939a6ca3fbd31600ae10a901f76260aaf27f611cdde646cf2c5df1f0</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>04_音视频翻译/本机重新生成产出/translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_174546.二维码.png</t>
+          <t>04_音视频翻译/本机重新生成产出/translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_194336.二维码.png</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: rebuild Yishu as an editorial translation studio
</commit_message>
<xml_diff>
--- a/collaboration/integration/final_outputs/ready_to_use/05_资源索引/统一交付资源索引.xlsx
+++ b/collaboration/integration/final_outputs/ready_to_use/05_资源索引/统一交付资源索引.xlsx
@@ -2251,7 +2251,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>DOCX_五套样例端到端验收_20260718_194336.json</t>
+          <t>DOCX_五套样例端到端验收_20260718_201706.json</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -2264,12 +2264,12 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>e3b1cd17bec39223987162d78b17f4a2aeb7a3c0e32ab66bcd1ccb01daefdafd</t>
+          <t>bc073f0731683c94dea205f9301e402e573bac60a5ee93d9e1573b310463edb2</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX_五套样例端到端验收_20260718_194336.json</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX_五套样例端到端验收_20260718_201706.json</t>
         </is>
       </c>
     </row>
@@ -2281,7 +2281,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试1_20260718_194336.docx</t>
+          <t>DOCX样例_测试1_20260718_201706.docx</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -2299,7 +2299,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试1_20260718_194336.docx</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试1_20260718_201706.docx</t>
         </is>
       </c>
     </row>
@@ -2311,7 +2311,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试1_20260718_194336.回填报告.json</t>
+          <t>DOCX样例_测试1_20260718_201706.回填报告.json</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -2324,12 +2324,12 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>62e78b877bf03de379bc58eb32c33515ff80a420e2019f3c56f0a8221a827096</t>
+          <t>5f971fd62b702e434f58cff26cab625bb8b1146e5266721dcad9a6283097e015</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试1_20260718_194336.回填报告.json</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试1_20260718_201706.回填报告.json</t>
         </is>
       </c>
     </row>
@@ -2341,7 +2341,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试2_20260718_194336.docx</t>
+          <t>DOCX样例_测试2_20260718_201706.docx</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -2359,7 +2359,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试2_20260718_194336.docx</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试2_20260718_201706.docx</t>
         </is>
       </c>
     </row>
@@ -2371,7 +2371,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试2_20260718_194336.回填报告.json</t>
+          <t>DOCX样例_测试2_20260718_201706.回填报告.json</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -2384,12 +2384,12 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>46ee547d2836fb99d84258402e50bdda4ae58cfe4e1c9ee5ca13c2e36d7ea076</t>
+          <t>ef746134003f068959b2b3f715b1ca29a30a6b5934535a612b779ec517fb1e12</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试2_20260718_194336.回填报告.json</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试2_20260718_201706.回填报告.json</t>
         </is>
       </c>
     </row>
@@ -2401,7 +2401,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试3_20260718_194336.docx</t>
+          <t>DOCX样例_测试3_20260718_201706.docx</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试3_20260718_194336.docx</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试3_20260718_201706.docx</t>
         </is>
       </c>
     </row>
@@ -2431,7 +2431,7 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试3_20260718_194336.回填报告.json</t>
+          <t>DOCX样例_测试3_20260718_201706.回填报告.json</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -2444,12 +2444,12 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>b94b1d90644287c1a88c33a5c58797f3fb6fcab57c5e84eb7f7d39185400cd4f</t>
+          <t>1d275ead3e779e037da35b2d8b873cf6388c83bf2e8fd53bb419d1ec5eda0def</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试3_20260718_194336.回填报告.json</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试3_20260718_201706.回填报告.json</t>
         </is>
       </c>
     </row>
@@ -2461,7 +2461,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试4_20260718_194336.docx</t>
+          <t>DOCX样例_测试4_20260718_201706.docx</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -2479,7 +2479,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试4_20260718_194336.docx</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试4_20260718_201706.docx</t>
         </is>
       </c>
     </row>
@@ -2491,7 +2491,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试4_20260718_194336.回填报告.json</t>
+          <t>DOCX样例_测试4_20260718_201706.回填报告.json</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -2504,12 +2504,12 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>76c97f70d0c3966a075e55cad784c198559f254d3dd78db40328ea8de054baaf</t>
+          <t>6681eb68c7829194237173be6f49b6d8dffa7fbd57fbb8bb77546b773cc418f0</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试4_20260718_194336.回填报告.json</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试4_20260718_201706.回填报告.json</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试5_20260718_194336.docx</t>
+          <t>DOCX样例_测试5_20260718_201706.docx</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -2539,7 +2539,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试5_20260718_194336.docx</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试5_20260718_201706.docx</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>DOCX样例_测试5_20260718_194336.回填报告.json</t>
+          <t>DOCX样例_测试5_20260718_201706.回填报告.json</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -2564,12 +2564,12 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>6d599971c03ef0c796f8e91dd3d11f928045711a8b5dcc7423f4d869c4ac2197</t>
+          <t>6c1262319d986858f43246d1a290eaca54195e687398cf11986ac2bd61048f0a</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试5_20260718_194336.回填报告.json</t>
+          <t>03_DOCX翻译/本机重新验收产出/DOCX样例_测试5_20260718_201706.回填报告.json</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_194336.txt</t>
+          <t>translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_201706.txt</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -2839,7 +2839,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>04_音视频翻译/本机重新生成产出/translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_194336.txt</t>
+          <t>04_音视频翻译/本机重新生成产出/translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_201706.txt</t>
         </is>
       </c>
     </row>
@@ -2851,7 +2851,7 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_194336.wav</t>
+          <t>translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_201706.wav</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -2869,7 +2869,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>04_音视频翻译/本机重新生成产出/translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_194336.wav</t>
+          <t>04_音视频翻译/本机重新生成产出/translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_201706.wav</t>
         </is>
       </c>
     </row>
@@ -2881,7 +2881,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_194336.二维码.png</t>
+          <t>translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_201706.二维码.png</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -2890,16 +2890,16 @@
         </is>
       </c>
       <c r="D82" s="2" t="n">
-        <v>2523</v>
+        <v>2606</v>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>b367e1b6939a6ca3fbd31600ae10a901f76260aaf27f611cdde646cf2c5df1f0</t>
+          <t>ccbbef69771bbb7163545515f73f97ec1fd197d8e6049569e40ff293c7ec7e85</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>04_音视频翻译/本机重新生成产出/translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_194336.二维码.png</t>
+          <t>04_音视频翻译/本机重新生成产出/translation_excel_411e8f80-8319-4798-85c9-210c828074a8_8d7754e3_英文配音_20260718_201706.二维码.png</t>
         </is>
       </c>
     </row>

</xml_diff>